<commit_message>
fix: refine pipeline in data transformation
</commit_message>
<xml_diff>
--- a/data/proteomics/ProMassRatio_across_compartment_cell_system_2018.xlsx
+++ b/data/proteomics/ProMassRatio_across_compartment_cell_system_2018.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AV140"/>
+  <dimension ref="A1:AW140"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -664,6 +664,11 @@
           <t>Mean Copy number - Glycerol</t>
         </is>
       </c>
+      <c r="AW1" s="1" t="inlineStr">
+        <is>
+          <t>MW_Kda</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
@@ -812,6 +817,9 @@
       <c r="AV2" t="n">
         <v>0.4618492745613613</v>
       </c>
+      <c r="AW2" t="n">
+        <v>0.1962093796106558</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
@@ -960,6 +968,9 @@
       <c r="AV3" t="n">
         <v>0.001122113969220753</v>
       </c>
+      <c r="AW3" t="n">
+        <v>0.005253104414995127</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
@@ -1108,6 +1119,9 @@
       <c r="AV4" t="n">
         <v>0.001292284076062277</v>
       </c>
+      <c r="AW4" t="n">
+        <v>0.0203838611442185</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
@@ -1256,6 +1270,9 @@
       <c r="AV5" t="n">
         <v>0.05417558567059665</v>
       </c>
+      <c r="AW5" t="n">
+        <v>0.02903842994648137</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
@@ -1404,6 +1421,9 @@
       <c r="AV6" t="n">
         <v>0.18172778009522</v>
       </c>
+      <c r="AW6" t="n">
+        <v>0.3095268237862273</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
@@ -1552,6 +1572,9 @@
       <c r="AV7" t="n">
         <v>0.5343268597243092</v>
       </c>
+      <c r="AW7" t="n">
+        <v>0.3142985903100214</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
@@ -1700,6 +1723,9 @@
       <c r="AV8" t="n">
         <v>0.275284843155997</v>
       </c>
+      <c r="AW8" t="n">
+        <v>0.1006287369862342</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
@@ -1848,6 +1874,9 @@
       <c r="AV9" t="n">
         <v>0.015100171413912</v>
       </c>
+      <c r="AW9" t="n">
+        <v>0.005878976001263633</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
@@ -1996,6 +2025,9 @@
       <c r="AV10" t="n">
         <v>0.01429139770097472</v>
       </c>
+      <c r="AW10" t="n">
+        <v>0.06251810833404513</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
@@ -2144,6 +2176,9 @@
       <c r="AV11" t="n">
         <v>0.01443239492252101</v>
       </c>
+      <c r="AW11" t="n">
+        <v>0.01364706967021041</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
@@ -2292,6 +2327,9 @@
       <c r="AV12" t="n">
         <v>0.03151205622048941</v>
       </c>
+      <c r="AW12" t="n">
+        <v>0.0905272573436209</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
@@ -2440,6 +2478,9 @@
       <c r="AV13" t="n">
         <v>0.001238101802164157</v>
       </c>
+      <c r="AW13" t="n">
+        <v>0.002260489701620927</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
@@ -2588,6 +2629,9 @@
       <c r="AV14" t="n">
         <v>0.02916914377367978</v>
       </c>
+      <c r="AW14" t="n">
+        <v>0.01123244399210152</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
@@ -2736,6 +2780,9 @@
       <c r="AV15" t="n">
         <v>0.01656651246356439</v>
       </c>
+      <c r="AW15" t="n">
+        <v>0.003013940397724772</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
@@ -2884,6 +2931,9 @@
       <c r="AV16" t="n">
         <v>0.004581542434239569</v>
       </c>
+      <c r="AW16" t="n">
+        <v>0.01804947997611915</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
@@ -3032,6 +3082,9 @@
       <c r="AV17" t="n">
         <v>0.006890812474675652</v>
       </c>
+      <c r="AW17" t="n">
+        <v>0.01706091903639325</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
@@ -3180,6 +3233,9 @@
       <c r="AV18" t="n">
         <v>0.005634766524365834</v>
       </c>
+      <c r="AW18" t="n">
+        <v>0.02480969836460922</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
@@ -3328,6 +3384,9 @@
       <c r="AV19" t="n">
         <v>0.006551882288010414</v>
       </c>
+      <c r="AW19" t="n">
+        <v>0.04882300598922126</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
@@ -3476,6 +3535,9 @@
       <c r="AV20" t="n">
         <v>0.01161634384306582</v>
       </c>
+      <c r="AW20" t="n">
+        <v>0.02888410256239034</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="1" t="n">
@@ -3624,6 +3686,9 @@
       <c r="AV21" t="n">
         <v>0.0003005603701137179</v>
       </c>
+      <c r="AW21" t="n">
+        <v>0.001659381317620119</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="1" t="n">
@@ -3772,6 +3837,9 @@
       <c r="AV22" t="n">
         <v>0.002056943430676889</v>
       </c>
+      <c r="AW22" t="n">
+        <v>0.01769556691146826</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="1" t="n">
@@ -3920,6 +3988,9 @@
       <c r="AV23" t="n">
         <v>0.02248113864497873</v>
       </c>
+      <c r="AW23" t="n">
+        <v>0.00949709137048602</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="1" t="n">
@@ -4068,6 +4139,9 @@
       <c r="AV24" t="n">
         <v>0.0001706354381370666</v>
       </c>
+      <c r="AW24" t="n">
+        <v>0.005611048830268917</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
@@ -4216,6 +4290,9 @@
       <c r="AV25" t="n">
         <v>0.005059549661378391</v>
       </c>
+      <c r="AW25" t="n">
+        <v>0.008530547090302593</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="1" t="n">
@@ -4364,6 +4441,9 @@
       <c r="AV26" t="n">
         <v>0.001999627641748845</v>
       </c>
+      <c r="AW26" t="n">
+        <v>0.01343387725475408</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="1" t="n">
@@ -4512,6 +4592,9 @@
       <c r="AV27" t="n">
         <v>0.01764598956663238</v>
       </c>
+      <c r="AW27" t="n">
+        <v>0.04513473910796071</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="1" t="n">
@@ -4660,6 +4743,9 @@
       <c r="AV28" t="n">
         <v>0.001137344503960974</v>
       </c>
+      <c r="AW28" t="n">
+        <v>0.008353011847097525</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="1" t="n">
@@ -4808,6 +4894,9 @@
       <c r="AV29" t="n">
         <v>0.01589416886557659</v>
       </c>
+      <c r="AW29" t="n">
+        <v>0.05716374935958042</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="1" t="n">
@@ -4956,6 +5045,9 @@
       <c r="AV30" t="n">
         <v>0.000109928444053154</v>
       </c>
+      <c r="AW30" t="n">
+        <v>0.001906311199661677</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="1" t="n">
@@ -5104,6 +5196,9 @@
       <c r="AV31" t="n">
         <v>1.238871306209699e-05</v>
       </c>
+      <c r="AW31" t="n">
+        <v>0.001776690721484506</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="1" t="n">
@@ -5252,6 +5347,9 @@
       <c r="AV32" t="n">
         <v>0.04899682016586929</v>
       </c>
+      <c r="AW32" t="n">
+        <v>0.02060340557110612</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="1" t="n">
@@ -5400,6 +5498,9 @@
       <c r="AV33" t="n">
         <v>0.02374151803376221</v>
       </c>
+      <c r="AW33" t="n">
+        <v>0.004869314656429779</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="1" t="n">
@@ -5548,6 +5649,9 @@
       <c r="AV34" t="n">
         <v>0.00253934263675869</v>
       </c>
+      <c r="AW34" t="n">
+        <v>0.01911108086869586</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="1" t="n">
@@ -5696,6 +5800,9 @@
       <c r="AV35" t="n">
         <v>0.001433399136245857</v>
       </c>
+      <c r="AW35" t="n">
+        <v>0.001807530489634456</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="1" t="n">
@@ -5844,6 +5951,9 @@
       <c r="AV36" t="n">
         <v>0.00205995660911744</v>
       </c>
+      <c r="AW36" t="n">
+        <v>0.007398015200117282</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="1" t="n">
@@ -5992,6 +6102,9 @@
       <c r="AV37" t="n">
         <v>0.02703481896938679</v>
       </c>
+      <c r="AW37" t="n">
+        <v>0.01147222705202277</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="1" t="n">
@@ -6140,6 +6253,9 @@
       <c r="AV38" t="n">
         <v>0.001464839110618275</v>
       </c>
+      <c r="AW38" t="n">
+        <v>0.009166751559561365</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="1" t="n">
@@ -6288,6 +6404,9 @@
       <c r="AV39" t="n">
         <v>0.000676666936049325</v>
       </c>
+      <c r="AW39" t="n">
+        <v>0.003320137204546559</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="1" t="n">
@@ -6436,6 +6555,9 @@
       <c r="AV40" t="n">
         <v>0.000621130604743151</v>
       </c>
+      <c r="AW40" t="n">
+        <v>0.002812862644857826</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="1" t="n">
@@ -6584,6 +6706,9 @@
       <c r="AV41" t="n">
         <v>0.001460083721304447</v>
       </c>
+      <c r="AW41" t="n">
+        <v>0.01118292853407937</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="1" t="n">
@@ -6732,6 +6857,9 @@
       <c r="AV42" t="n">
         <v>0.0004230703310083183</v>
       </c>
+      <c r="AW42" t="n">
+        <v>0.004087768952183323</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="1" t="n">
@@ -6880,6 +7008,9 @@
       <c r="AV43" t="n">
         <v>0.002386498855335299</v>
       </c>
+      <c r="AW43" t="n">
+        <v>0.01178072700523176</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="1" t="n">
@@ -7028,6 +7159,9 @@
       <c r="AV44" t="n">
         <v>0.003865998870593426</v>
       </c>
+      <c r="AW44" t="n">
+        <v>0.01862627074349292</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="1" t="n">
@@ -7176,6 +7310,9 @@
       <c r="AV45" t="n">
         <v>0.0001175043227099133</v>
       </c>
+      <c r="AW45" t="n">
+        <v>0.001473590214124054</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="1" t="n">
@@ -7324,6 +7461,9 @@
       <c r="AV46" t="n">
         <v>0.0002468002506297721</v>
       </c>
+      <c r="AW46" t="n">
+        <v>0.003334352346649306</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="1" t="n">
@@ -7472,6 +7612,9 @@
       <c r="AV47" t="n">
         <v>0.0009730048791857368</v>
       </c>
+      <c r="AW47" t="n">
+        <v>0.004231294317002064</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="1" t="n">
@@ -7620,6 +7763,9 @@
       <c r="AV48" t="n">
         <v>0.001397300040994695</v>
       </c>
+      <c r="AW48" t="n">
+        <v>0.005257793901270202</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="1" t="n">
@@ -7768,6 +7914,9 @@
       <c r="AV49" t="n">
         <v>0.006185061005938767</v>
       </c>
+      <c r="AW49" t="n">
+        <v>0.000344202162543321</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="1" t="n">
@@ -7916,6 +8065,9 @@
       <c r="AV50" t="n">
         <v>0.001543343671939363</v>
       </c>
+      <c r="AW50" t="n">
+        <v>0.008072466473904067</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="1" t="n">
@@ -8064,6 +8216,9 @@
       <c r="AV51" t="n">
         <v>0.03241689537255583</v>
       </c>
+      <c r="AW51" t="n">
+        <v>0.01515135609678211</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="1" t="n">
@@ -8212,6 +8367,9 @@
       <c r="AV52" t="n">
         <v>0.001635704170342016</v>
       </c>
+      <c r="AW52" t="n">
+        <v>0.009405850618783436</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="1" t="n">
@@ -8360,6 +8518,9 @@
       <c r="AV53" t="n">
         <v>0.0001800987522364393</v>
       </c>
+      <c r="AW53" t="n">
+        <v>0.003790308401205325</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="1" t="n">
@@ -8508,6 +8669,9 @@
       <c r="AV54" t="n">
         <v>0.03192106773616282</v>
       </c>
+      <c r="AW54" t="n">
+        <v>0.04577103490241575</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="1" t="n">
@@ -8656,6 +8820,9 @@
       <c r="AV55" t="n">
         <v>0.01159043826818307</v>
       </c>
+      <c r="AW55" t="n">
+        <v>0.01424361304542963</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="1" t="n">
@@ -8804,6 +8971,9 @@
       <c r="AV56" t="n">
         <v>0.01044666036935426</v>
       </c>
+      <c r="AW56" t="n">
+        <v>0.01276548941103365</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="1" t="n">
@@ -8952,6 +9122,9 @@
       <c r="AV57" t="n">
         <v>0.001011309178873485</v>
       </c>
+      <c r="AW57" t="n">
+        <v>0.00168681046499978</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="1" t="n">
@@ -9100,6 +9273,9 @@
       <c r="AV58" t="n">
         <v>0.001069752073132918</v>
       </c>
+      <c r="AW58" t="n">
+        <v>0.0103214595217978</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="1" t="n">
@@ -9248,6 +9424,9 @@
       <c r="AV59" t="n">
         <v>0.001909625276334307</v>
       </c>
+      <c r="AW59" t="n">
+        <v>0.01045173585249723</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="1" t="n">
@@ -9396,6 +9575,9 @@
       <c r="AV60" t="n">
         <v>0.004130988529073322</v>
       </c>
+      <c r="AW60" t="n">
+        <v>0.005058648989885182</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="1" t="n">
@@ -9544,6 +9726,9 @@
       <c r="AV61" t="n">
         <v>0.0007184560479033581</v>
       </c>
+      <c r="AW61" t="n">
+        <v>0.00601417450983403</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="1" t="n">
@@ -9692,6 +9877,9 @@
       <c r="AV62" t="n">
         <v>0.000178944052380501</v>
       </c>
+      <c r="AW62" t="n">
+        <v>0.001776827396521334</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="1" t="n">
@@ -9840,6 +10028,9 @@
       <c r="AV63" t="n">
         <v>0.008699833413839066</v>
       </c>
+      <c r="AW63" t="n">
+        <v>0.01109248030993588</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="1" t="n">
@@ -9988,6 +10179,9 @@
       <c r="AV64" t="n">
         <v>0.0003502283016611317</v>
       </c>
+      <c r="AW64" t="n">
+        <v>0.004198159534160469</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="1" t="n">
@@ -10136,6 +10330,9 @@
       <c r="AV65" t="n">
         <v>0.06695954156479796</v>
       </c>
+      <c r="AW65" t="n">
+        <v>0.004053001887837817</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="1" t="n">
@@ -10284,6 +10481,9 @@
       <c r="AV66" t="n">
         <v>0.001726964604881934</v>
       </c>
+      <c r="AW66" t="n">
+        <v>0.006944242193060264</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="1" t="n">
@@ -10432,6 +10632,9 @@
       <c r="AV67" t="n">
         <v>7.353145269273597e-05</v>
       </c>
+      <c r="AW67" t="n">
+        <v>0.002560803539466176</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="1" t="n">
@@ -10580,6 +10783,9 @@
       <c r="AV68" t="n">
         <v>0.001009819567614193</v>
       </c>
+      <c r="AW68" t="n">
+        <v>0.006683211638168775</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="1" t="n">
@@ -10728,6 +10934,9 @@
       <c r="AV69" t="n">
         <v>0.0007979041247192996</v>
       </c>
+      <c r="AW69" t="n">
+        <v>0.002097312530705863</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="1" t="n">
@@ -10876,6 +11085,9 @@
       <c r="AV70" t="n">
         <v>0.0002209157430782023</v>
       </c>
+      <c r="AW70" t="n">
+        <v>0.0009197742076836608</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="1" t="n">
@@ -11024,6 +11236,9 @@
       <c r="AV71" t="n">
         <v>0.008862215564604335</v>
       </c>
+      <c r="AW71" t="n">
+        <v>0.003985532584302741</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="1" t="n">
@@ -11172,6 +11387,9 @@
       <c r="AV72" t="n">
         <v>0.007652309409213573</v>
       </c>
+      <c r="AW72" t="n">
+        <v>0.001448548032147315</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="1" t="n">
@@ -11320,6 +11538,9 @@
       <c r="AV73" t="n">
         <v>0.01300198452152243</v>
       </c>
+      <c r="AW73" t="n">
+        <v>0.01080310641742983</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="1" t="n">
@@ -11468,6 +11689,9 @@
       <c r="AV74" t="n">
         <v>0.003921438784907996</v>
       </c>
+      <c r="AW74" t="n">
+        <v>0.002276573257156201</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="1" t="n">
@@ -11616,6 +11840,9 @@
       <c r="AV75" t="n">
         <v>6.629596832265301e-05</v>
       </c>
+      <c r="AW75" t="n">
+        <v>0.0008611625099106528</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="1" t="n">
@@ -11764,6 +11991,9 @@
       <c r="AV76" t="n">
         <v>0.003044407142924511</v>
       </c>
+      <c r="AW76" t="n">
+        <v>0.006572137681007484</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="1" t="n">
@@ -11912,6 +12142,9 @@
       <c r="AV77" t="n">
         <v>0.0002851402655445836</v>
       </c>
+      <c r="AW77" t="n">
+        <v>0.004350580661158885</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="1" t="n">
@@ -12060,6 +12293,9 @@
       <c r="AV78" t="n">
         <v>0.0008072129491922994</v>
       </c>
+      <c r="AW78" t="n">
+        <v>0.001413915766293509</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="1" t="n">
@@ -12208,6 +12444,9 @@
       <c r="AV79" t="n">
         <v>0.0001072628928871379</v>
       </c>
+      <c r="AW79" t="n">
+        <v>0.002641441498437574</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="1" t="n">
@@ -12356,6 +12595,9 @@
       <c r="AV80" t="n">
         <v>0.0002623222740790311</v>
       </c>
+      <c r="AW80" t="n">
+        <v>0.001988165785391115</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="1" t="n">
@@ -12504,6 +12746,9 @@
       <c r="AV81" t="n">
         <v>0.0001396303701552319</v>
       </c>
+      <c r="AW81" t="n">
+        <v>0.004297523224207481</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="1" t="n">
@@ -12652,6 +12897,9 @@
       <c r="AV82" t="n">
         <v>0.00036948768057208</v>
       </c>
+      <c r="AW82" t="n">
+        <v>0.0007003138187420178</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="1" t="n">
@@ -12800,6 +13048,9 @@
       <c r="AV83" t="n">
         <v>0.006460582241480924</v>
       </c>
+      <c r="AW83" t="n">
+        <v>0.001024541409426986</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="1" t="n">
@@ -12948,6 +13199,9 @@
       <c r="AV84" t="n">
         <v>0.00185562093987605</v>
       </c>
+      <c r="AW84" t="n">
+        <v>0.004705033451464358</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="1" t="n">
@@ -13096,6 +13350,9 @@
       <c r="AV85" t="n">
         <v>0.0001378674688484711</v>
       </c>
+      <c r="AW85" t="n">
+        <v>0.006499312404919338</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="1" t="n">
@@ -13244,6 +13501,9 @@
       <c r="AV86" t="n">
         <v>0.001042144243643991</v>
       </c>
+      <c r="AW86" t="n">
+        <v>0.003207667097809976</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="1" t="n">
@@ -13392,6 +13652,9 @@
       <c r="AV87" t="n">
         <v>0.000272864231417742</v>
       </c>
+      <c r="AW87" t="n">
+        <v>0.001709803772454175</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="1" t="n">
@@ -13540,6 +13803,9 @@
       <c r="AV88" t="n">
         <v>0.002839220281627605</v>
       </c>
+      <c r="AW88" t="n">
+        <v>0.00200826170716775</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="1" t="n">
@@ -13688,6 +13954,9 @@
       <c r="AV89" t="n">
         <v>5.347254431217515e-05</v>
       </c>
+      <c r="AW89" t="n">
+        <v>0.0009027999187275902</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="1" t="n">
@@ -13836,6 +14105,9 @@
       <c r="AV90" t="n">
         <v>0.0009393562783724216</v>
       </c>
+      <c r="AW90" t="n">
+        <v>0.001206818682170717</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="1" t="n">
@@ -13984,6 +14256,9 @@
       <c r="AV91" t="n">
         <v>5.158569747307589e-05</v>
       </c>
+      <c r="AW91" t="n">
+        <v>0.00194369416791573</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="1" t="n">
@@ -14132,6 +14407,9 @@
       <c r="AV92" t="n">
         <v>0.000373211629191225</v>
       </c>
+      <c r="AW92" t="n">
+        <v>0.000973637620767577</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="1" t="n">
@@ -14280,6 +14558,9 @@
       <c r="AV93" t="n">
         <v>0.004569225170636796</v>
       </c>
+      <c r="AW93" t="n">
+        <v>0.001242628792849915</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="1" t="n">
@@ -14428,6 +14709,9 @@
       <c r="AV94" t="n">
         <v>0.0007510576491312458</v>
       </c>
+      <c r="AW94" t="n">
+        <v>0.002814724490382405</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="1" t="n">
@@ -14576,6 +14860,9 @@
       <c r="AV95" t="n">
         <v>0.005850690977811756</v>
       </c>
+      <c r="AW95" t="n">
+        <v>0.001535217519917891</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="1" t="n">
@@ -14724,6 +15011,9 @@
       <c r="AV96" t="n">
         <v>0.001425335401138262</v>
       </c>
+      <c r="AW96" t="n">
+        <v>0.001979974665907034</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="1" t="n">
@@ -14872,6 +15162,9 @@
       <c r="AV97" t="n">
         <v>0.0001935209527461194</v>
       </c>
+      <c r="AW97" t="n">
+        <v>0.001057753130618833</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="1" t="n">
@@ -15020,6 +15313,9 @@
       <c r="AV98" t="n">
         <v>0.0006873583118329203</v>
       </c>
+      <c r="AW98" t="n">
+        <v>0.003278323400487581</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="1" t="n">
@@ -15168,6 +15464,9 @@
       <c r="AV99" t="n">
         <v>0.0007367234093583091</v>
       </c>
+      <c r="AW99" t="n">
+        <v>0.0004898520892045732</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="1" t="n">
@@ -15316,6 +15615,9 @@
       <c r="AV100" t="n">
         <v>0.0005438225516457441</v>
       </c>
+      <c r="AW100" t="n">
+        <v>0.001950931376959701</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="1" t="n">
@@ -15464,6 +15766,9 @@
       <c r="AV101" t="n">
         <v>0.0003178279291376699</v>
       </c>
+      <c r="AW101" t="n">
+        <v>0.002143437384439088</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="1" t="n">
@@ -15612,6 +15917,9 @@
       <c r="AV102" t="n">
         <v>0.006186789203150737</v>
       </c>
+      <c r="AW102" t="n">
+        <v>0.003817434799304321</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="1" t="n">
@@ -15760,6 +16068,9 @@
       <c r="AV103" t="n">
         <v>0.00015495276352063</v>
       </c>
+      <c r="AW103" t="n">
+        <v>0.004044102685325407</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="1" t="n">
@@ -15908,6 +16219,9 @@
       <c r="AV104" t="n">
         <v>0.0003424803261544606</v>
       </c>
+      <c r="AW104" t="n">
+        <v>0.002720073743424572</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="1" t="n">
@@ -16056,6 +16370,9 @@
       <c r="AV105" t="n">
         <v>0.0009381612738827193</v>
       </c>
+      <c r="AW105" t="n">
+        <v>0.001088699236326041</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="1" t="n">
@@ -16204,6 +16521,9 @@
       <c r="AV106" t="n">
         <v>0.001497868049242571</v>
       </c>
+      <c r="AW106" t="n">
+        <v>0.001819343028458214</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="1" t="n">
@@ -16352,6 +16672,9 @@
       <c r="AV107" t="n">
         <v>0.001348956743185075</v>
       </c>
+      <c r="AW107" t="n">
+        <v>0.001108737610718749</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="1" t="n">
@@ -16500,6 +16823,9 @@
       <c r="AV108" t="n">
         <v>0.002584622160016889</v>
       </c>
+      <c r="AW108" t="n">
+        <v>0.01480593324163297</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="1" t="n">
@@ -16648,6 +16974,9 @@
       <c r="AV109" t="n">
         <v>0.0001049314519787276</v>
       </c>
+      <c r="AW109" t="n">
+        <v>0.00149429444927971</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="1" t="n">
@@ -16796,6 +17125,9 @@
       <c r="AV110" t="n">
         <v>0.0007361041695121767</v>
       </c>
+      <c r="AW110" t="n">
+        <v>0.0009422511524703116</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="1" t="n">
@@ -16944,6 +17276,9 @@
       <c r="AV111" t="n">
         <v>0.004905374768465229</v>
       </c>
+      <c r="AW111" t="n">
+        <v>0.003568668717854935</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="1" t="n">
@@ -17092,6 +17427,9 @@
       <c r="AV112" t="n">
         <v>0.001142311248496796</v>
       </c>
+      <c r="AW112" t="n">
+        <v>0.003819095541742674</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="1" t="n">
@@ -17240,6 +17578,9 @@
       <c r="AV113" t="n">
         <v>0.0004590480566516545</v>
       </c>
+      <c r="AW113" t="n">
+        <v>0.0007596160851221599</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="1" t="n">
@@ -17388,6 +17729,9 @@
       <c r="AV114" t="n">
         <v>0.000270604338619106</v>
       </c>
+      <c r="AW114" t="n">
+        <v>0.003493768608370171</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="1" t="n">
@@ -17536,6 +17880,9 @@
       <c r="AV115" t="n">
         <v>0.002258915063934394</v>
       </c>
+      <c r="AW115" t="n">
+        <v>0.001938936500500998</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="1" t="n">
@@ -17684,6 +18031,9 @@
       <c r="AV116" t="n">
         <v>0.000228648035440099</v>
       </c>
+      <c r="AW116" t="n">
+        <v>0.002959983470141973</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="1" t="n">
@@ -17832,6 +18182,9 @@
       <c r="AV117" t="n">
         <v>0.0006090506934280426</v>
       </c>
+      <c r="AW117" t="n">
+        <v>0.00240222546790252</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="1" t="n">
@@ -17980,6 +18333,9 @@
       <c r="AV118" t="n">
         <v>4.358867311810457e-05</v>
       </c>
+      <c r="AW118" t="n">
+        <v>0.002032278044474471</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="1" t="n">
@@ -18128,6 +18484,9 @@
       <c r="AV119" t="n">
         <v>0.002172018414940078</v>
       </c>
+      <c r="AW119" t="n">
+        <v>0.002419611032999162</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="1" t="n">
@@ -18276,6 +18635,9 @@
       <c r="AV120" t="n">
         <v>0.08360284627616985</v>
       </c>
+      <c r="AW120" t="n">
+        <v>0.00660292490589385</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="1" t="n">
@@ -18424,6 +18786,9 @@
       <c r="AV121" t="n">
         <v>2.854546006385735e-05</v>
       </c>
+      <c r="AW121" t="n">
+        <v>0.00123285324376269</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="1" t="n">
@@ -18572,6 +18937,9 @@
       <c r="AV122" t="n">
         <v>8.125319837815005e-05</v>
       </c>
+      <c r="AW122" t="n">
+        <v>0.002451317452240765</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="1" t="n">
@@ -18720,6 +19088,9 @@
       <c r="AV123" t="n">
         <v>0.00233420342455888</v>
       </c>
+      <c r="AW123" t="n">
+        <v>0.001829679039023692</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="1" t="n">
@@ -18868,6 +19239,9 @@
       <c r="AV124" t="n">
         <v>0.000386058694041086</v>
       </c>
+      <c r="AW124" t="n">
+        <v>0.003288167756229503</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="1" t="n">
@@ -19016,6 +19390,9 @@
       <c r="AV125" t="n">
         <v>0.001517542937346934</v>
       </c>
+      <c r="AW125" t="n">
+        <v>0.000757008312909168</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="1" t="n">
@@ -19164,6 +19541,9 @@
       <c r="AV126" t="n">
         <v>0.001304681710415026</v>
       </c>
+      <c r="AW126" t="n">
+        <v>0.002697109522419662</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="1" t="n">
@@ -19312,6 +19692,9 @@
       <c r="AV127" t="n">
         <v>0.0004974689503453524</v>
       </c>
+      <c r="AW127" t="n">
+        <v>0.002541810087952289</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="1" t="n">
@@ -19460,6 +19843,9 @@
       <c r="AV128" t="n">
         <v>0.0001529168630063303</v>
       </c>
+      <c r="AW128" t="n">
+        <v>0.0008887411553855175</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="1" t="n">
@@ -19608,6 +19994,9 @@
       <c r="AV129" t="n">
         <v>0.0005552908144132834</v>
       </c>
+      <c r="AW129" t="n">
+        <v>0.002324939644044921</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="1" t="n">
@@ -19756,6 +20145,9 @@
       <c r="AV130" t="n">
         <v>0.0006356016970868021</v>
       </c>
+      <c r="AW130" t="n">
+        <v>0.00200135226800615</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="1" t="n">
@@ -19904,6 +20296,9 @@
       <c r="AV131" t="n">
         <v>0.0003964474303155096</v>
       </c>
+      <c r="AW131" t="n">
+        <v>0.0008390812033885059</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="1" t="n">
@@ -20052,6 +20447,9 @@
       <c r="AV132" t="n">
         <v>0.0003567687296194612</v>
       </c>
+      <c r="AW132" t="n">
+        <v>0.001524464916333978</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="1" t="n">
@@ -20200,6 +20598,9 @@
       <c r="AV133" t="n">
         <v>0.007939335256427295</v>
       </c>
+      <c r="AW133" t="n">
+        <v>0.002925566068705333</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="1" t="n">
@@ -20348,6 +20749,9 @@
       <c r="AV134" t="n">
         <v>0.0001449993142983505</v>
       </c>
+      <c r="AW134" t="n">
+        <v>0.001680161552853462</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="1" t="n">
@@ -20496,6 +20900,9 @@
       <c r="AV135" t="n">
         <v>0.0001346735478659551</v>
       </c>
+      <c r="AW135" t="n">
+        <v>0.001166680007396074</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="1" t="n">
@@ -20644,6 +21051,9 @@
       <c r="AV136" t="n">
         <v>3.406979674286824e-05</v>
       </c>
+      <c r="AW136" t="n">
+        <v>0.001471176038816776</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="1" t="n">
@@ -20792,6 +21202,9 @@
       <c r="AV137" t="n">
         <v>0.0001377576194572109</v>
       </c>
+      <c r="AW137" t="n">
+        <v>0.001077716755963939</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="1" t="n">
@@ -20940,6 +21353,9 @@
       <c r="AV138" t="n">
         <v>0.0001262936839268749</v>
       </c>
+      <c r="AW138" t="n">
+        <v>0.003986688536101638</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="1" t="n">
@@ -21088,6 +21504,9 @@
       <c r="AV139" t="n">
         <v>0.0001538333761116757</v>
       </c>
+      <c r="AW139" t="n">
+        <v>0.003004179860998572</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="1" t="n">
@@ -21235,6 +21654,9 @@
       </c>
       <c r="AV140" t="n">
         <v>2.98514171291593e-05</v>
+      </c>
+      <c r="AW140" t="n">
+        <v>0.0009960413802942328</v>
       </c>
     </row>
   </sheetData>

</xml_diff>